<commit_message>
Added as_base_R to the package, a function that converts everything back to its base type. Updated documentation to reflect this.
</commit_message>
<xml_diff>
--- a/tests/testthat/_output_excel_snaps/data_to_worksheet_data_table.xlsx
+++ b/tests/testthat/_output_excel_snaps/data_to_worksheet_data_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">mpg</t>
   </si>
@@ -47,6 +47,9 @@
     <t xml:space="preserve">carb</t>
   </si>
   <si>
+    <t xml:space="preserve">scientific</t>
+  </si>
+  <si>
     <t xml:space="preserve">test</t>
   </si>
 </sst>
@@ -54,7 +57,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="0"/>
@@ -65,6 +68,7 @@
     <numFmt numFmtId="172" formatCode="0.00"/>
     <numFmt numFmtId="173" formatCode="0.00"/>
     <numFmt numFmtId="174" formatCode="0.00"/>
+    <numFmt numFmtId="175" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -100,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -135,6 +139,9 @@
     <xf numFmtId="174" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="175" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -144,9 +151,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="table_test_1" displayName="table_test_1" ref="A2:K34" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A2:K34"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="table_test_1" displayName="table_test_1" ref="A2:L34" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A2:L34"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="mpg"/>
     <tableColumn id="2" name="cyl"/>
     <tableColumn id="3" name="disp"/>
@@ -158,6 +165,7 @@
     <tableColumn id="9" name="am"/>
     <tableColumn id="10" name="gear"/>
     <tableColumn id="11" name="carb"/>
+    <tableColumn id="12" name="scientific"/>
   </tableColumns>
   <tableStyleInfo name="none" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -479,6 +487,9 @@
       <c r="K2" t="s">
         <v>10</v>
       </c>
+      <c r="L2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -503,7 +514,7 @@
         <v>16.46</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I3" s="9" t="n">
         <v>1</v>
@@ -513,6 +524,9 @@
       </c>
       <c r="K3" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>16.46</v>
       </c>
     </row>
     <row r="4">
@@ -538,7 +552,7 @@
         <v>17.02</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I4" s="9" t="n">
         <v>1</v>
@@ -548,6 +562,9 @@
       </c>
       <c r="K4" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="5">
@@ -573,7 +590,7 @@
         <v>18.61</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I5" s="9" t="n">
         <v>1</v>
@@ -583,6 +600,9 @@
       </c>
       <c r="K5" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>18.61</v>
       </c>
     </row>
     <row r="6">
@@ -608,7 +628,7 @@
         <v>19.44</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>0</v>
@@ -618,6 +638,9 @@
       </c>
       <c r="K6" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>19.44</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +666,7 @@
         <v>17.02</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I7" s="9" t="n">
         <v>0</v>
@@ -653,6 +676,9 @@
       </c>
       <c r="K7" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="8">
@@ -678,7 +704,7 @@
         <v>20.22</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>0</v>
@@ -688,6 +714,9 @@
       </c>
       <c r="K8" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>20.22</v>
       </c>
     </row>
     <row r="9">
@@ -713,7 +742,7 @@
         <v>15.84</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I9" s="9" t="n">
         <v>0</v>
@@ -723,6 +752,9 @@
       </c>
       <c r="K9" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>15.84</v>
       </c>
     </row>
     <row r="10">
@@ -748,7 +780,7 @@
         <v>20</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>0</v>
@@ -758,6 +790,9 @@
       </c>
       <c r="K10" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -783,7 +818,7 @@
         <v>22.9</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I11" s="9" t="n">
         <v>0</v>
@@ -793,6 +828,9 @@
       </c>
       <c r="K11" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>22.9</v>
       </c>
     </row>
     <row r="12">
@@ -818,7 +856,7 @@
         <v>18.3</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I12" s="9" t="n">
         <v>0</v>
@@ -828,6 +866,9 @@
       </c>
       <c r="K12" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>18.3</v>
       </c>
     </row>
     <row r="13">
@@ -853,7 +894,7 @@
         <v>18.9</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I13" s="9" t="n">
         <v>0</v>
@@ -863,6 +904,9 @@
       </c>
       <c r="K13" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>18.9</v>
       </c>
     </row>
     <row r="14">
@@ -888,7 +932,7 @@
         <v>17.4</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I14" s="9" t="n">
         <v>0</v>
@@ -898,6 +942,9 @@
       </c>
       <c r="K14" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>17.4</v>
       </c>
     </row>
     <row r="15">
@@ -923,7 +970,7 @@
         <v>17.6</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I15" s="9" t="n">
         <v>0</v>
@@ -933,6 +980,9 @@
       </c>
       <c r="K15" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>17.6</v>
       </c>
     </row>
     <row r="16">
@@ -958,7 +1008,7 @@
         <v>18</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I16" s="9" t="n">
         <v>0</v>
@@ -968,6 +1018,9 @@
       </c>
       <c r="K16" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -993,7 +1046,7 @@
         <v>17.98</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I17" s="9" t="n">
         <v>0</v>
@@ -1003,6 +1056,9 @@
       </c>
       <c r="K17" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>17.98</v>
       </c>
     </row>
     <row r="18">
@@ -1028,7 +1084,7 @@
         <v>17.82</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I18" s="9" t="n">
         <v>0</v>
@@ -1038,6 +1094,9 @@
       </c>
       <c r="K18" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>17.82</v>
       </c>
     </row>
     <row r="19">
@@ -1063,7 +1122,7 @@
         <v>17.42</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I19" s="9" t="n">
         <v>0</v>
@@ -1073,6 +1132,9 @@
       </c>
       <c r="K19" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>17.42</v>
       </c>
     </row>
     <row r="20">
@@ -1098,7 +1160,7 @@
         <v>19.47</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I20" s="9" t="n">
         <v>1</v>
@@ -1108,6 +1170,9 @@
       </c>
       <c r="K20" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>19.47</v>
       </c>
     </row>
     <row r="21">
@@ -1133,7 +1198,7 @@
         <v>18.52</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I21" s="9" t="n">
         <v>1</v>
@@ -1143,6 +1208,9 @@
       </c>
       <c r="K21" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>18.52</v>
       </c>
     </row>
     <row r="22">
@@ -1168,7 +1236,7 @@
         <v>19.9</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I22" s="9" t="n">
         <v>1</v>
@@ -1178,6 +1246,9 @@
       </c>
       <c r="K22" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>19.9</v>
       </c>
     </row>
     <row r="23">
@@ -1203,7 +1274,7 @@
         <v>20.01</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>0</v>
@@ -1213,6 +1284,9 @@
       </c>
       <c r="K23" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>20.01</v>
       </c>
     </row>
     <row r="24">
@@ -1238,7 +1312,7 @@
         <v>16.87</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I24" s="9" t="n">
         <v>0</v>
@@ -1248,6 +1322,9 @@
       </c>
       <c r="K24" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>16.87</v>
       </c>
     </row>
     <row r="25">
@@ -1273,7 +1350,7 @@
         <v>17.3</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I25" s="9" t="n">
         <v>0</v>
@@ -1283,6 +1360,9 @@
       </c>
       <c r="K25" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L25" s="12" t="n">
+        <v>17.3</v>
       </c>
     </row>
     <row r="26">
@@ -1308,7 +1388,7 @@
         <v>15.41</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I26" s="9" t="n">
         <v>0</v>
@@ -1318,6 +1398,9 @@
       </c>
       <c r="K26" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L26" s="12" t="n">
+        <v>15.41</v>
       </c>
     </row>
     <row r="27">
@@ -1343,7 +1426,7 @@
         <v>17.05</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I27" s="9" t="n">
         <v>0</v>
@@ -1353,6 +1436,9 @@
       </c>
       <c r="K27" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>17.05</v>
       </c>
     </row>
     <row r="28">
@@ -1378,7 +1464,7 @@
         <v>18.9</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I28" s="9" t="n">
         <v>1</v>
@@ -1388,6 +1474,9 @@
       </c>
       <c r="K28" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>18.9</v>
       </c>
     </row>
     <row r="29">
@@ -1413,7 +1502,7 @@
         <v>16.7</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I29" s="9" t="n">
         <v>1</v>
@@ -1423,6 +1512,9 @@
       </c>
       <c r="K29" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>16.7</v>
       </c>
     </row>
     <row r="30">
@@ -1448,7 +1540,7 @@
         <v>16.9</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I30" s="9" t="n">
         <v>1</v>
@@ -1458,6 +1550,9 @@
       </c>
       <c r="K30" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L30" s="12" t="n">
+        <v>16.9</v>
       </c>
     </row>
     <row r="31">
@@ -1483,7 +1578,7 @@
         <v>14.5</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I31" s="9" t="n">
         <v>1</v>
@@ -1493,6 +1588,9 @@
       </c>
       <c r="K31" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L31" s="12" t="n">
+        <v>14.5</v>
       </c>
     </row>
     <row r="32">
@@ -1518,7 +1616,7 @@
         <v>15.5</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I32" s="9" t="n">
         <v>1</v>
@@ -1528,6 +1626,9 @@
       </c>
       <c r="K32" s="11" t="n">
         <v>6</v>
+      </c>
+      <c r="L32" s="12" t="n">
+        <v>15.5</v>
       </c>
     </row>
     <row r="33">
@@ -1553,7 +1654,7 @@
         <v>14.6</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I33" s="9" t="n">
         <v>1</v>
@@ -1563,6 +1664,9 @@
       </c>
       <c r="K33" s="11" t="n">
         <v>8</v>
+      </c>
+      <c r="L33" s="12" t="n">
+        <v>14.6</v>
       </c>
     </row>
     <row r="34">
@@ -1588,7 +1692,7 @@
         <v>18.6</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I34" s="9" t="n">
         <v>1</v>
@@ -1598,6 +1702,9 @@
       </c>
       <c r="K34" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L34" s="12" t="n">
+        <v>18.6</v>
       </c>
     </row>
     <row r="35">
@@ -1612,6 +1719,7 @@
       <c r="I35" s="9"/>
       <c r="J35" s="10"/>
       <c r="K35" s="11"/>
+      <c r="L35" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>